<commit_message>
feat: flujo de auditoría Drive por estudiante (backend + frontend)
</commit_message>
<xml_diff>
--- a/docs/students/10a.xlsx
+++ b/docs/students/10a.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\María Alexandra\Listados Actualizados\LISTADOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\AgenteIA_Alexandra\docs\students\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3198465-D7D3-4BC1-A76A-ADBF788287FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C23807-A2DF-4A24-A1D6-459063F32E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="93">
   <si>
     <t xml:space="preserve">CORREO MAMÁ </t>
   </si>
@@ -48,21 +48,6 @@
     <t>eddgonzalez@hotmail.com</t>
   </si>
   <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Correo institucional</t>
-  </si>
-  <si>
-    <t>Nombre mamá</t>
-  </si>
-  <si>
-    <t>Nombre papá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORREO PAPÁ </t>
-  </si>
-  <si>
     <t>carolinacarranzao@gmail.com</t>
   </si>
   <si>
@@ -310,6 +295,27 @@
   </si>
   <si>
     <t>23AC0309@cac.edu.co</t>
+  </si>
+  <si>
+    <t>NOMBRE</t>
+  </si>
+  <si>
+    <t>CORREO INSTITUCIONAL</t>
+  </si>
+  <si>
+    <t>NOMBRE MAMÁ</t>
+  </si>
+  <si>
+    <t>NOMBRE  PAPÁ</t>
+  </si>
+  <si>
+    <t>CORREO PAPÁ</t>
+  </si>
+  <si>
+    <t>ID_DRIVE</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1odLpbR5jpl2Qf17hE0nwNbIF1OdTgv3o?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -361,7 +367,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -384,33 +390,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -420,9 +406,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -436,18 +419,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -789,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="30.75" customWidth="1"/>
@@ -798,60 +775,82 @@
     <col min="4" max="4" width="28.75" customWidth="1"/>
     <col min="5" max="5" width="30.875" customWidth="1"/>
     <col min="6" max="6" width="27.375" customWidth="1"/>
+    <col min="7" max="7" width="78.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="71.45" customHeight="1">
-      <c r="A1" s="16"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-    </row>
-    <row r="2" spans="1:6" ht="15">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
+    <row r="1" spans="1:7" ht="15">
+      <c r="A1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B2" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="9" t="s">
+      <c r="D2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.5">
+      <c r="A3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="15" t="s">
+      <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="28.5">
-      <c r="A4" s="5" t="s">
+      <c r="G3" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>77</v>
+      <c r="B4" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>16</v>
@@ -865,13 +864,16 @@
       <c r="F4" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>78</v>
+      <c r="B5" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>21</v>
@@ -882,91 +884,107 @@
       <c r="E5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>79</v>
+      <c r="B6" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="B7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1"/>
+      <c r="G7" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="G8" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
+      <c r="B9" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="E9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>83</v>
+      <c r="B10" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>42</v>
@@ -980,13 +998,16 @@
       <c r="F10" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>84</v>
+      <c r="B11" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>47</v>
@@ -997,172 +1018,182 @@
       <c r="E11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="1"/>
+      <c r="G11" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>87</v>
+      <c r="B14" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="B16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="F16" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="G16" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7">
+      <c r="F17" s="12"/>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="6:7">
+      <c r="F18" s="12"/>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="6:7">
+      <c r="F19" s="12"/>
+      <c r="G19" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="F16" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="D16" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="B13" r:id="rId3" display="23ac0321@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
-    <hyperlink ref="F13" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
-    <hyperlink ref="D17" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
-    <hyperlink ref="F17" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
-    <hyperlink ref="B3" r:id="rId7" display="26AC0020@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
-    <hyperlink ref="C4" r:id="rId8" display="mailto:lilin7lilon@gmail.com" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
-    <hyperlink ref="E4" r:id="rId9" display="ZENSEYLEE@GMAIL.COM" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
-    <hyperlink ref="D4" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
-    <hyperlink ref="F4" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
-    <hyperlink ref="B4" r:id="rId12" display="mailto:23AC0312@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
-    <hyperlink ref="D5" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
-    <hyperlink ref="F5" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
-    <hyperlink ref="B5" r:id="rId15" display="mailto:24AC0505@Australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
-    <hyperlink ref="D6" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
-    <hyperlink ref="F6" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
-    <hyperlink ref="B7" r:id="rId18" display="23ac0315@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
-    <hyperlink ref="F7" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
-    <hyperlink ref="D7" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
-    <hyperlink ref="D10" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
-    <hyperlink ref="F10" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
-    <hyperlink ref="D11" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
-    <hyperlink ref="F11" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
-    <hyperlink ref="B11" r:id="rId25" display="mailto:24AC0506@Australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
-    <hyperlink ref="D12" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
-    <hyperlink ref="B8" r:id="rId27" display="23AC0317@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
-    <hyperlink ref="D8" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
-    <hyperlink ref="B9" r:id="rId29" display="26AC0619@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
-    <hyperlink ref="B15" r:id="rId30" display="26AC0021@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
-    <hyperlink ref="D15" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
-    <hyperlink ref="F15" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
-    <hyperlink ref="D9" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
-    <hyperlink ref="F9" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
-    <hyperlink ref="D3" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
-    <hyperlink ref="F3" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
+    <hyperlink ref="F15" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="D15" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="B12" r:id="rId3" display="23ac0321@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
+    <hyperlink ref="F12" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="D16" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
+    <hyperlink ref="F16" r:id="rId6" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
+    <hyperlink ref="B2" r:id="rId7" display="26AC0020@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
+    <hyperlink ref="C3" r:id="rId8" display="mailto:lilin7lilon@gmail.com" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="E3" r:id="rId9" display="ZENSEYLEE@GMAIL.COM" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="D3" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
+    <hyperlink ref="F3" r:id="rId11" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="B3" r:id="rId12" display="mailto:23AC0312@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
+    <hyperlink ref="D4" r:id="rId13" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="F4" r:id="rId14" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
+    <hyperlink ref="B4" r:id="rId15" display="mailto:24AC0505@Australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="D5" r:id="rId16" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
+    <hyperlink ref="F5" r:id="rId17" xr:uid="{00000000-0004-0000-0400-000010000000}"/>
+    <hyperlink ref="B6" r:id="rId18" display="23ac0315@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000011000000}"/>
+    <hyperlink ref="F6" r:id="rId19" xr:uid="{00000000-0004-0000-0400-000012000000}"/>
+    <hyperlink ref="D6" r:id="rId20" xr:uid="{00000000-0004-0000-0400-000013000000}"/>
+    <hyperlink ref="D9" r:id="rId21" xr:uid="{00000000-0004-0000-0400-000014000000}"/>
+    <hyperlink ref="F9" r:id="rId22" xr:uid="{00000000-0004-0000-0400-000015000000}"/>
+    <hyperlink ref="D10" r:id="rId23" xr:uid="{00000000-0004-0000-0400-000016000000}"/>
+    <hyperlink ref="F10" r:id="rId24" xr:uid="{00000000-0004-0000-0400-000017000000}"/>
+    <hyperlink ref="B10" r:id="rId25" display="mailto:24AC0506@Australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-000018000000}"/>
+    <hyperlink ref="D11" r:id="rId26" xr:uid="{00000000-0004-0000-0400-000019000000}"/>
+    <hyperlink ref="B7" r:id="rId27" display="23AC0317@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001A000000}"/>
+    <hyperlink ref="D7" r:id="rId28" xr:uid="{00000000-0004-0000-0400-00001B000000}"/>
+    <hyperlink ref="B8" r:id="rId29" display="26AC0619@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001C000000}"/>
+    <hyperlink ref="B14" r:id="rId30" display="26AC0021@australianocampestre.edu.co" xr:uid="{00000000-0004-0000-0400-00001D000000}"/>
+    <hyperlink ref="D14" r:id="rId31" xr:uid="{00000000-0004-0000-0400-00001E000000}"/>
+    <hyperlink ref="F14" r:id="rId32" xr:uid="{00000000-0004-0000-0400-00001F000000}"/>
+    <hyperlink ref="D8" r:id="rId33" xr:uid="{00000000-0004-0000-0400-000020000000}"/>
+    <hyperlink ref="F8" r:id="rId34" xr:uid="{00000000-0004-0000-0400-000021000000}"/>
+    <hyperlink ref="D2" r:id="rId35" xr:uid="{00000000-0004-0000-0400-000022000000}"/>
+    <hyperlink ref="F2" r:id="rId36" xr:uid="{00000000-0004-0000-0400-000023000000}"/>
+    <hyperlink ref="G2" r:id="rId37" xr:uid="{51CBC6EE-EC42-4719-8EFF-83E99B96C7C7}"/>
+    <hyperlink ref="G3:G13" r:id="rId38" display="https://drive.google.com/drive/folders/1odLpbR5jpl2Qf17hE0nwNbIF1OdTgv3o?usp=drive_link" xr:uid="{BBAF923C-8E1A-49FB-A7D4-E09B2FC45652}"/>
+    <hyperlink ref="G14:G19" r:id="rId39" display="https://drive.google.com/drive/folders/1odLpbR5jpl2Qf17hE0nwNbIF1OdTgv3o?usp=drive_link" xr:uid="{1FB5CC92-1939-4900-9BA9-D3266F8D45B8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId40"/>
 </worksheet>
 </file>
 

</xml_diff>